<commit_message>
feat: strengthen roster financial workflows
</commit_message>
<xml_diff>
--- a/sample-data/manchester-city-squad.xlsx
+++ b/sample-data/manchester-city-squad.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Squad" sheetId="1" r:id="rId1"/>
+    <sheet name="Manchester City squad" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:M24"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="21.83203125" customWidth="1"/>
+    <col min="8" max="8" width="27.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
+    <col min="13" max="13" width="27.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,361 +451,418 @@
       <c r="L1" t="str">
         <v>contract_end</v>
       </c>
+      <c r="M1" t="str">
+        <v>amortisation_treatment</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Ederson</v>
+        <v>Gianluigi Donnarumma</v>
       </c>
       <c r="B2" t="str">
         <v>GK</v>
       </c>
-      <c r="C2">
-        <v>31</v>
+      <c r="C2" t="str">
+        <v>25</v>
       </c>
       <c r="D2" t="str">
-        <v>Brazil</v>
+        <v>Italy</v>
       </c>
       <c r="E2" t="str">
-        <v>1993-08-17</v>
+        <v>1999-02-25</v>
       </c>
       <c r="F2" t="str">
-        <v>2017-07-01</v>
-      </c>
-      <c r="G2">
-        <v>35000000</v>
-      </c>
-      <c r="I2">
-        <v>200000</v>
-      </c>
-      <c r="J2">
-        <v>2800000</v>
+        <v>2025-09-01</v>
+      </c>
+      <c r="G2" t="str">
+        <v>26000000</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v>250000</v>
+      </c>
+      <c r="J2" t="str">
+        <v>2500000</v>
       </c>
       <c r="K2" t="str">
-        <v>2023-07-01</v>
+        <v>2025-09-01</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-06-30</v>
+        <v>2030-06-30</v>
+      </c>
+      <c r="M2" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Stefan Ortega</v>
+        <v>Marcus Bettinelli</v>
       </c>
       <c r="B3" t="str">
         <v>GK</v>
       </c>
-      <c r="C3">
-        <v>18</v>
+      <c r="C3" t="str">
+        <v>13</v>
       </c>
       <c r="D3" t="str">
-        <v>Germany</v>
+        <v>England</v>
       </c>
       <c r="E3" t="str">
-        <v>1992-11-06</v>
+        <v>1992-05-24</v>
       </c>
       <c r="F3" t="str">
-        <v>2022-07-01</v>
-      </c>
-      <c r="G3">
+        <v>2025-06-10</v>
+      </c>
+      <c r="G3" t="str">
         <v>0</v>
       </c>
-      <c r="I3">
-        <v>60000</v>
-      </c>
-      <c r="J3">
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>45000</v>
+      </c>
+      <c r="J3" t="str">
         <v>0</v>
       </c>
       <c r="K3" t="str">
-        <v>2024-07-01</v>
+        <v>2025-06-10</v>
       </c>
       <c r="L3" t="str">
         <v>2027-06-30</v>
       </c>
+      <c r="M3" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Kyle Walker</v>
+        <v>Ruben Dias</v>
       </c>
       <c r="B4" t="str">
         <v>DEF</v>
       </c>
-      <c r="C4">
-        <v>2</v>
+      <c r="C4" t="str">
+        <v>3</v>
       </c>
       <c r="D4" t="str">
-        <v>England</v>
+        <v>Portugal</v>
       </c>
       <c r="E4" t="str">
-        <v>1990-05-28</v>
+        <v>1997-05-14</v>
       </c>
       <c r="F4" t="str">
-        <v>2017-07-14</v>
-      </c>
-      <c r="G4">
-        <v>45000000</v>
-      </c>
-      <c r="I4">
-        <v>160000</v>
-      </c>
-      <c r="J4">
-        <v>3600000</v>
+        <v>2020-09-29</v>
+      </c>
+      <c r="G4" t="str">
+        <v>62000000</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>280000</v>
+      </c>
+      <c r="J4" t="str">
+        <v>5000000</v>
       </c>
       <c r="K4" t="str">
-        <v>2023-07-01</v>
+        <v>2025-07-01</v>
       </c>
       <c r="L4" t="str">
-        <v>2026-06-30</v>
+        <v>2029-06-30</v>
+      </c>
+      <c r="M4" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Ruben Dias</v>
+        <v>Josko Gvardiol</v>
       </c>
       <c r="B5" t="str">
         <v>DEF</v>
       </c>
-      <c r="C5">
-        <v>3</v>
+      <c r="C5" t="str">
+        <v>24</v>
       </c>
       <c r="D5" t="str">
-        <v>Portugal</v>
+        <v>Croatia</v>
       </c>
       <c r="E5" t="str">
-        <v>1997-05-14</v>
+        <v>2002-01-23</v>
       </c>
       <c r="F5" t="str">
-        <v>2020-09-29</v>
-      </c>
-      <c r="G5">
-        <v>62000000</v>
-      </c>
-      <c r="H5">
-        <v>31000000</v>
-      </c>
-      <c r="I5">
+        <v>2023-08-05</v>
+      </c>
+      <c r="G5" t="str">
+        <v>77000000</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
         <v>200000</v>
       </c>
-      <c r="J5">
-        <v>5000000</v>
+      <c r="J5" t="str">
+        <v>6100000</v>
       </c>
       <c r="K5" t="str">
-        <v>2023-07-01</v>
+        <v>2023-08-05</v>
       </c>
       <c r="L5" t="str">
-        <v>2027-06-30</v>
+        <v>2028-06-30</v>
+      </c>
+      <c r="M5" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>John Stones</v>
+        <v>Marc Guehi</v>
       </c>
       <c r="B6" t="str">
         <v>DEF</v>
       </c>
-      <c r="C6">
-        <v>5</v>
+      <c r="C6" t="str">
+        <v/>
       </c>
       <c r="D6" t="str">
         <v>England</v>
       </c>
       <c r="E6" t="str">
-        <v>1994-05-28</v>
+        <v>2000-07-13</v>
       </c>
       <c r="F6" t="str">
-        <v>2016-08-09</v>
-      </c>
-      <c r="G6">
-        <v>47500000</v>
-      </c>
-      <c r="I6">
-        <v>250000</v>
-      </c>
-      <c r="J6">
-        <v>3800000</v>
+        <v>2026-01-20</v>
+      </c>
+      <c r="G6" t="str">
+        <v>30000000</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v>180000</v>
+      </c>
+      <c r="J6" t="str">
+        <v>4000000</v>
       </c>
       <c r="K6" t="str">
-        <v>2022-09-01</v>
+        <v>2026-01-20</v>
       </c>
       <c r="L6" t="str">
-        <v>2026-06-30</v>
+        <v>2031-06-30</v>
+      </c>
+      <c r="M6" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Nathan Ake</v>
+        <v>Abdukodir Khusanov</v>
       </c>
       <c r="B7" t="str">
         <v>DEF</v>
       </c>
-      <c r="C7">
-        <v>6</v>
+      <c r="C7" t="str">
+        <v>45</v>
       </c>
       <c r="D7" t="str">
-        <v>Netherlands</v>
+        <v>Uzbekistan</v>
       </c>
       <c r="E7" t="str">
-        <v>1995-02-18</v>
+        <v>2004-02-29</v>
       </c>
       <c r="F7" t="str">
-        <v>2020-08-05</v>
-      </c>
-      <c r="G7">
-        <v>41000000</v>
-      </c>
-      <c r="I7">
-        <v>120000</v>
-      </c>
-      <c r="J7">
-        <v>3200000</v>
+        <v>2025-01-20</v>
+      </c>
+      <c r="G7" t="str">
+        <v>33000000</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>70000</v>
+      </c>
+      <c r="J7" t="str">
+        <v>2000000</v>
       </c>
       <c r="K7" t="str">
-        <v>2023-07-01</v>
+        <v>2025-01-20</v>
       </c>
       <c r="L7" t="str">
-        <v>2027-06-30</v>
+        <v>2029-06-30</v>
+      </c>
+      <c r="M7" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Manuel Akanji</v>
+        <v>Rayan Ait-Nouri</v>
       </c>
       <c r="B8" t="str">
         <v>DEF</v>
       </c>
-      <c r="C8">
-        <v>25</v>
+      <c r="C8" t="str">
+        <v>21</v>
       </c>
       <c r="D8" t="str">
-        <v>Switzerland</v>
+        <v>Algeria</v>
       </c>
       <c r="E8" t="str">
-        <v>1995-07-19</v>
+        <v>2001-06-06</v>
       </c>
       <c r="F8" t="str">
-        <v>2022-09-01</v>
-      </c>
-      <c r="G8">
-        <v>15000000</v>
-      </c>
-      <c r="I8">
+        <v>2025-06-09</v>
+      </c>
+      <c r="G8" t="str">
+        <v>31800000</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
         <v>110000</v>
       </c>
-      <c r="J8">
-        <v>1200000</v>
+      <c r="J8" t="str">
+        <v>3000000</v>
       </c>
       <c r="K8" t="str">
-        <v>2022-09-01</v>
+        <v>2025-06-09</v>
       </c>
       <c r="L8" t="str">
-        <v>2027-06-30</v>
+        <v>2030-06-30</v>
+      </c>
+      <c r="M8" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Josko Gvardiol</v>
+        <v>Rico Lewis</v>
       </c>
       <c r="B9" t="str">
         <v>DEF</v>
       </c>
-      <c r="C9">
-        <v>24</v>
+      <c r="C9" t="str">
+        <v>82</v>
       </c>
       <c r="D9" t="str">
-        <v>Croatia</v>
+        <v>England</v>
       </c>
       <c r="E9" t="str">
-        <v>2002-01-23</v>
+        <v>2004-11-21</v>
       </c>
       <c r="F9" t="str">
-        <v>2023-08-05</v>
-      </c>
-      <c r="G9">
-        <v>77000000</v>
-      </c>
-      <c r="H9">
-        <v>57000000</v>
-      </c>
-      <c r="I9">
-        <v>140000</v>
-      </c>
-      <c r="J9">
-        <v>6100000</v>
+        <v>2022-07-01</v>
+      </c>
+      <c r="G9" t="str">
+        <v>0</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v>80000</v>
+      </c>
+      <c r="J9" t="str">
+        <v>0</v>
       </c>
       <c r="K9" t="str">
-        <v>2023-08-05</v>
+        <v>2025-07-01</v>
       </c>
       <c r="L9" t="str">
-        <v>2028-06-30</v>
+        <v>2030-06-30</v>
+      </c>
+      <c r="M9" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Rico Lewis</v>
+        <v>Matheus Nunes</v>
       </c>
       <c r="B10" t="str">
-        <v>DEF</v>
-      </c>
-      <c r="C10">
-        <v>82</v>
+        <v>MID</v>
+      </c>
+      <c r="C10" t="str">
+        <v>27</v>
       </c>
       <c r="D10" t="str">
-        <v>England</v>
+        <v>Portugal</v>
       </c>
       <c r="E10" t="str">
-        <v>2004-11-21</v>
+        <v>1998-08-27</v>
       </c>
       <c r="F10" t="str">
-        <v>2020-07-01</v>
-      </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-      <c r="I10">
-        <v>40000</v>
-      </c>
-      <c r="J10">
-        <v>0</v>
+        <v>2023-09-01</v>
+      </c>
+      <c r="G10" t="str">
+        <v>53000000</v>
+      </c>
+      <c r="H10" t="str">
+        <v>40000000</v>
+      </c>
+      <c r="I10" t="str">
+        <v>80000</v>
+      </c>
+      <c r="J10" t="str">
+        <v>4200000</v>
       </c>
       <c r="K10" t="str">
-        <v>2023-07-01</v>
+        <v>2023-09-01</v>
       </c>
       <c r="L10" t="str">
         <v>2028-06-30</v>
       </c>
+      <c r="M10" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Kevin De Bruyne</v>
+        <v>Nico O'Reilly</v>
       </c>
       <c r="B11" t="str">
         <v>MID</v>
       </c>
-      <c r="C11">
-        <v>17</v>
+      <c r="C11" t="str">
+        <v>75</v>
       </c>
       <c r="D11" t="str">
-        <v>Belgium</v>
+        <v>England</v>
       </c>
       <c r="E11" t="str">
-        <v>1991-06-28</v>
+        <v>2005-03-21</v>
       </c>
       <c r="F11" t="str">
-        <v>2015-08-30</v>
-      </c>
-      <c r="G11">
-        <v>55000000</v>
-      </c>
-      <c r="I11">
-        <v>400000</v>
-      </c>
-      <c r="J11">
-        <v>4400000</v>
+        <v>2024-07-01</v>
+      </c>
+      <c r="G11" t="str">
+        <v>0</v>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v>50000</v>
+      </c>
+      <c r="J11" t="str">
+        <v>0</v>
       </c>
       <c r="K11" t="str">
-        <v>2023-07-01</v>
+        <v>2024-07-01</v>
       </c>
       <c r="L11" t="str">
-        <v>2027-06-30</v>
+        <v>2030-06-30</v>
+      </c>
+      <c r="M11" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="12">
@@ -800,7 +872,7 @@
       <c r="B12" t="str">
         <v>MID</v>
       </c>
-      <c r="C12">
+      <c r="C12" t="str">
         <v>16</v>
       </c>
       <c r="D12" t="str">
@@ -812,13 +884,16 @@
       <c r="F12" t="str">
         <v>2019-07-04</v>
       </c>
-      <c r="G12">
+      <c r="G12" t="str">
         <v>62800000</v>
       </c>
-      <c r="I12">
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
         <v>220000</v>
       </c>
-      <c r="J12">
+      <c r="J12" t="str">
         <v>5000000</v>
       </c>
       <c r="K12" t="str">
@@ -827,373 +902,418 @@
       <c r="L12" t="str">
         <v>2027-06-30</v>
       </c>
+      <c r="M12" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Bernardo Silva</v>
+        <v>Nico Gonzalez</v>
       </c>
       <c r="B13" t="str">
         <v>MID</v>
       </c>
-      <c r="C13">
-        <v>20</v>
+      <c r="C13" t="str">
+        <v>14</v>
       </c>
       <c r="D13" t="str">
-        <v>Portugal</v>
+        <v>Spain</v>
       </c>
       <c r="E13" t="str">
-        <v>1994-08-10</v>
+        <v>2002-01-03</v>
       </c>
       <c r="F13" t="str">
-        <v>2017-05-26</v>
-      </c>
-      <c r="G13">
-        <v>43000000</v>
-      </c>
-      <c r="I13">
-        <v>200000</v>
-      </c>
-      <c r="J13">
-        <v>3400000</v>
+        <v>2025-02-03</v>
+      </c>
+      <c r="G13" t="str">
+        <v>50000000</v>
+      </c>
+      <c r="H13" t="str">
+        <v>42000000</v>
+      </c>
+      <c r="I13" t="str">
+        <v>90000</v>
+      </c>
+      <c r="J13" t="str">
+        <v>4000000</v>
       </c>
       <c r="K13" t="str">
-        <v>2023-07-01</v>
+        <v>2025-02-03</v>
       </c>
       <c r="L13" t="str">
-        <v>2026-06-30</v>
+        <v>2029-06-30</v>
+      </c>
+      <c r="M13" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Mateo Kovacic</v>
+        <v>Tijjani Reijnders</v>
       </c>
       <c r="B14" t="str">
         <v>MID</v>
       </c>
-      <c r="C14">
-        <v>8</v>
+      <c r="C14" t="str">
+        <v>4</v>
       </c>
       <c r="D14" t="str">
-        <v>Croatia</v>
+        <v>Netherlands</v>
       </c>
       <c r="E14" t="str">
-        <v>1994-05-06</v>
+        <v>1998-07-29</v>
       </c>
       <c r="F14" t="str">
-        <v>2023-06-27</v>
-      </c>
-      <c r="G14">
-        <v>25000000</v>
-      </c>
-      <c r="H14">
-        <v>15000000</v>
-      </c>
-      <c r="I14">
-        <v>120000</v>
-      </c>
-      <c r="J14">
-        <v>2000000</v>
+        <v>2025-06-10</v>
+      </c>
+      <c r="G14" t="str">
+        <v>46000000</v>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v>150000</v>
+      </c>
+      <c r="J14" t="str">
+        <v>3000000</v>
       </c>
       <c r="K14" t="str">
-        <v>2023-06-27</v>
+        <v>2025-06-10</v>
       </c>
       <c r="L14" t="str">
-        <v>2027-06-30</v>
+        <v>2030-06-30</v>
+      </c>
+      <c r="M14" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Matheus Nunes</v>
+        <v>Elliot Anderson</v>
       </c>
       <c r="B15" t="str">
         <v>MID</v>
       </c>
-      <c r="C15">
-        <v>27</v>
+      <c r="C15" t="str">
+        <v/>
       </c>
       <c r="D15" t="str">
-        <v>Portugal</v>
+        <v>England</v>
       </c>
       <c r="E15" t="str">
-        <v>1998-08-27</v>
+        <v>2002-11-06</v>
       </c>
       <c r="F15" t="str">
-        <v>2023-09-01</v>
-      </c>
-      <c r="G15">
-        <v>53000000</v>
-      </c>
-      <c r="H15">
-        <v>40000000</v>
-      </c>
-      <c r="I15">
-        <v>80000</v>
-      </c>
-      <c r="J15">
-        <v>4200000</v>
+        <v>2026-07-01</v>
+      </c>
+      <c r="G15" t="str">
+        <v>116000000</v>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v>200000</v>
+      </c>
+      <c r="J15" t="str">
+        <v>10000000</v>
       </c>
       <c r="K15" t="str">
-        <v>2023-09-01</v>
+        <v>2026-07-01</v>
       </c>
       <c r="L15" t="str">
-        <v>2028-06-30</v>
+        <v>2031-06-30</v>
+      </c>
+      <c r="M15" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Ilkay Gundogan</v>
+        <v>Phil Foden</v>
       </c>
       <c r="B16" t="str">
         <v>MID</v>
       </c>
-      <c r="C16">
-        <v>19</v>
+      <c r="C16" t="str">
+        <v>47</v>
       </c>
       <c r="D16" t="str">
-        <v>Germany</v>
+        <v>England</v>
       </c>
       <c r="E16" t="str">
-        <v>1990-10-24</v>
+        <v>2000-05-28</v>
       </c>
       <c r="F16" t="str">
-        <v>2023-08-21</v>
-      </c>
-      <c r="G16">
+        <v>2017-07-01</v>
+      </c>
+      <c r="G16" t="str">
         <v>0</v>
       </c>
-      <c r="I16">
-        <v>200000</v>
-      </c>
-      <c r="J16">
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v>225000</v>
+      </c>
+      <c r="J16" t="str">
         <v>0</v>
       </c>
       <c r="K16" t="str">
-        <v>2024-07-01</v>
+        <v>2022-07-01</v>
       </c>
       <c r="L16" t="str">
-        <v>2026-06-30</v>
+        <v>2027-06-30</v>
+      </c>
+      <c r="M16" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Nico Gonzalez</v>
+        <v>Rayan Cherki</v>
       </c>
       <c r="B17" t="str">
         <v>MID</v>
       </c>
-      <c r="C17">
-        <v>14</v>
+      <c r="C17" t="str">
+        <v>10</v>
       </c>
       <c r="D17" t="str">
-        <v>Spain</v>
+        <v>France</v>
       </c>
       <c r="E17" t="str">
-        <v>2002-01-03</v>
+        <v>2003-08-17</v>
       </c>
       <c r="F17" t="str">
-        <v>2025-01-31</v>
-      </c>
-      <c r="G17">
-        <v>50000000</v>
-      </c>
-      <c r="H17">
-        <v>42000000</v>
-      </c>
-      <c r="I17">
-        <v>90000</v>
-      </c>
-      <c r="J17">
-        <v>4000000</v>
+        <v>2025-06-10</v>
+      </c>
+      <c r="G17" t="str">
+        <v>36500000</v>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v>150000</v>
+      </c>
+      <c r="J17" t="str">
+        <v>3000000</v>
       </c>
       <c r="K17" t="str">
-        <v>2025-01-31</v>
+        <v>2025-06-10</v>
       </c>
       <c r="L17" t="str">
-        <v>2029-06-30</v>
+        <v>2030-06-30</v>
+      </c>
+      <c r="M17" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Phil Foden</v>
+        <v>Jeremy Doku</v>
       </c>
       <c r="B18" t="str">
         <v>FWD</v>
       </c>
-      <c r="C18">
-        <v>47</v>
+      <c r="C18" t="str">
+        <v>11</v>
       </c>
       <c r="D18" t="str">
-        <v>England</v>
+        <v>Belgium</v>
       </c>
       <c r="E18" t="str">
-        <v>2000-05-28</v>
+        <v>2002-05-27</v>
       </c>
       <c r="F18" t="str">
-        <v>2017-07-01</v>
-      </c>
-      <c r="G18">
-        <v>0</v>
-      </c>
-      <c r="I18">
-        <v>225000</v>
-      </c>
-      <c r="J18">
-        <v>0</v>
+        <v>2023-08-24</v>
+      </c>
+      <c r="G18" t="str">
+        <v>55500000</v>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v>100000</v>
+      </c>
+      <c r="J18" t="str">
+        <v>4400000</v>
       </c>
       <c r="K18" t="str">
-        <v>2024-07-01</v>
+        <v>2023-08-24</v>
       </c>
       <c r="L18" t="str">
-        <v>2027-06-30</v>
+        <v>2028-06-30</v>
+      </c>
+      <c r="M18" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Jack Grealish</v>
+        <v>Antoine Semenyo</v>
       </c>
       <c r="B19" t="str">
         <v>FWD</v>
       </c>
-      <c r="C19">
-        <v>10</v>
+      <c r="C19" t="str">
+        <v/>
       </c>
       <c r="D19" t="str">
-        <v>England</v>
+        <v>Ghana</v>
       </c>
       <c r="E19" t="str">
-        <v>1995-09-10</v>
+        <v>2000-01-07</v>
       </c>
       <c r="F19" t="str">
-        <v>2021-08-05</v>
-      </c>
-      <c r="G19">
-        <v>100000000</v>
-      </c>
-      <c r="H19">
-        <v>33000000</v>
-      </c>
-      <c r="I19">
-        <v>300000</v>
-      </c>
-      <c r="J19">
-        <v>8000000</v>
+        <v>2026-01-09</v>
+      </c>
+      <c r="G19" t="str">
+        <v>64000000</v>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v>160000</v>
+      </c>
+      <c r="J19" t="str">
+        <v>5000000</v>
       </c>
       <c r="K19" t="str">
-        <v>2021-08-05</v>
+        <v>2026-01-09</v>
       </c>
       <c r="L19" t="str">
-        <v>2027-06-30</v>
+        <v>2031-06-30</v>
+      </c>
+      <c r="M19" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Jeremy Doku</v>
+        <v>Erling Haaland</v>
       </c>
       <c r="B20" t="str">
         <v>FWD</v>
       </c>
-      <c r="C20">
-        <v>11</v>
+      <c r="C20" t="str">
+        <v>9</v>
       </c>
       <c r="D20" t="str">
-        <v>Belgium</v>
+        <v>Norway</v>
       </c>
       <c r="E20" t="str">
-        <v>2002-05-27</v>
+        <v>2000-07-21</v>
       </c>
       <c r="F20" t="str">
-        <v>2023-08-31</v>
-      </c>
-      <c r="G20">
-        <v>55500000</v>
-      </c>
-      <c r="H20">
-        <v>42000000</v>
-      </c>
-      <c r="I20">
-        <v>100000</v>
-      </c>
-      <c r="J20">
-        <v>4400000</v>
+        <v>2022-07-01</v>
+      </c>
+      <c r="G20" t="str">
+        <v>51000000</v>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v>375000</v>
+      </c>
+      <c r="J20" t="str">
+        <v>4100000</v>
       </c>
       <c r="K20" t="str">
-        <v>2023-08-31</v>
+        <v>2025-07-01</v>
       </c>
       <c r="L20" t="str">
-        <v>2028-06-30</v>
+        <v>2034-06-30</v>
+      </c>
+      <c r="M20" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Savinho</v>
+        <v>Omar Marmoush</v>
       </c>
       <c r="B21" t="str">
         <v>FWD</v>
       </c>
-      <c r="C21">
-        <v>26</v>
+      <c r="C21" t="str">
+        <v>7</v>
       </c>
       <c r="D21" t="str">
-        <v>Brazil</v>
+        <v>Egypt</v>
       </c>
       <c r="E21" t="str">
-        <v>2004-04-10</v>
+        <v>1999-02-07</v>
       </c>
       <c r="F21" t="str">
-        <v>2024-07-01</v>
-      </c>
-      <c r="G21">
-        <v>21000000</v>
-      </c>
-      <c r="H21">
-        <v>17000000</v>
-      </c>
-      <c r="I21">
-        <v>70000</v>
-      </c>
-      <c r="J21">
-        <v>1700000</v>
+        <v>2025-01-31</v>
+      </c>
+      <c r="G21" t="str">
+        <v>59000000</v>
+      </c>
+      <c r="H21" t="str">
+        <v>50000000</v>
+      </c>
+      <c r="I21" t="str">
+        <v>150000</v>
+      </c>
+      <c r="J21" t="str">
+        <v>4700000</v>
       </c>
       <c r="K21" t="str">
-        <v>2024-07-01</v>
+        <v>2025-01-31</v>
       </c>
       <c r="L21" t="str">
         <v>2029-06-30</v>
       </c>
+      <c r="M21" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Erling Haaland</v>
+        <v>Savinho</v>
       </c>
       <c r="B22" t="str">
         <v>FWD</v>
       </c>
-      <c r="C22">
-        <v>9</v>
+      <c r="C22" t="str">
+        <v>26</v>
       </c>
       <c r="D22" t="str">
-        <v>Norway</v>
+        <v>Brazil</v>
       </c>
       <c r="E22" t="str">
-        <v>2000-07-21</v>
+        <v>2004-04-10</v>
       </c>
       <c r="F22" t="str">
-        <v>2022-07-01</v>
-      </c>
-      <c r="G22">
-        <v>51000000</v>
-      </c>
-      <c r="I22">
-        <v>375000</v>
-      </c>
-      <c r="J22">
-        <v>4100000</v>
+        <v>2024-07-18</v>
+      </c>
+      <c r="G22" t="str">
+        <v>21000000</v>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v>80000</v>
+      </c>
+      <c r="J22" t="str">
+        <v>1500000</v>
       </c>
       <c r="K22" t="str">
-        <v>2024-01-01</v>
+        <v>2024-07-18</v>
       </c>
       <c r="L22" t="str">
-        <v>2033-06-30</v>
+        <v>2029-06-30</v>
+      </c>
+      <c r="M22" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
     <row r="23">
@@ -1203,7 +1323,7 @@
       <c r="B23" t="str">
         <v>FWD</v>
       </c>
-      <c r="C23">
+      <c r="C23" t="str">
         <v>52</v>
       </c>
       <c r="D23" t="str">
@@ -1213,15 +1333,18 @@
         <v>2003-07-12</v>
       </c>
       <c r="F23" t="str">
-        <v>2020-07-01</v>
-      </c>
-      <c r="G23">
+        <v>2023-07-01</v>
+      </c>
+      <c r="G23" t="str">
         <v>0</v>
       </c>
-      <c r="I23">
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
         <v>30000</v>
       </c>
-      <c r="J23">
+      <c r="J23" t="str">
         <v>0</v>
       </c>
       <c r="K23" t="str">
@@ -1230,48 +1353,54 @@
       <c r="L23" t="str">
         <v>2029-06-30</v>
       </c>
+      <c r="M23" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Omar Marmoush</v>
+        <v>Jeremy Monga</v>
       </c>
       <c r="B24" t="str">
         <v>FWD</v>
       </c>
-      <c r="C24">
-        <v>7</v>
+      <c r="C24" t="str">
+        <v/>
       </c>
       <c r="D24" t="str">
-        <v>Egypt</v>
+        <v>England</v>
       </c>
       <c r="E24" t="str">
-        <v>1999-02-07</v>
+        <v>2009-07-10</v>
       </c>
       <c r="F24" t="str">
-        <v>2025-01-31</v>
-      </c>
-      <c r="G24">
-        <v>59000000</v>
-      </c>
-      <c r="H24">
-        <v>50000000</v>
-      </c>
-      <c r="I24">
-        <v>150000</v>
-      </c>
-      <c r="J24">
-        <v>4700000</v>
+        <v>2026-07-01</v>
+      </c>
+      <c r="G24" t="str">
+        <v>10000000</v>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v>20000</v>
+      </c>
+      <c r="J24" t="str">
+        <v>500000</v>
       </c>
       <c r="K24" t="str">
-        <v>2025-01-31</v>
+        <v>2026-07-01</v>
       </c>
       <c r="L24" t="str">
-        <v>2029-06-30</v>
+        <v>2031-06-30</v>
+      </c>
+      <c r="M24" t="str">
+        <v>CONTINUE_CURRENT_SCHEDULE</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>